<commit_message>
updated tag template, added --list-template flag
</commit_message>
<xml_diff>
--- a/ww_tag_template.xlsx
+++ b/ww_tag_template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\wwtags\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F73B65-7279-43C8-A365-C062CBEABA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B64BE1-4456-41F1-A7EA-F93B90B64798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9345" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20970" yWindow="-15705" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEVICE_LIST" sheetId="9" r:id="rId1"/>
-    <sheet name="MADE" sheetId="3" r:id="rId2"/>
-    <sheet name="NEED TO MAKE" sheetId="8" r:id="rId3"/>
+    <sheet name="$MADE" sheetId="3" r:id="rId2"/>
+    <sheet name="$NEED TO MAKE" sheetId="8" r:id="rId3"/>
     <sheet name="Device Template" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>

</xml_diff>

<commit_message>
add OFFSET column support for Step 7 PLC addressing
- Add optional OFFSET column to DEVICE_LIST
- Support OFFSET+N arithmetic notation in templates for byte-addressed types (BOOL, INT, REAL, etc.)
- --force flag added but disabled (commented out)
- Update tag template workbook
</commit_message>
<xml_diff>
--- a/ww_tag_template.xlsx
+++ b/ww_tag_template.xlsx
@@ -1,34 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\wwtags\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\wwtags\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B64BE1-4456-41F1-A7EA-F93B90B64798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCE7247-BA9C-4AB6-A54B-C63A44EFDB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20970" yWindow="-15705" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEVICE_LIST" sheetId="9" r:id="rId1"/>
     <sheet name="$MADE" sheetId="3" r:id="rId2"/>
     <sheet name="$NEED TO MAKE" sheetId="8" r:id="rId3"/>
     <sheet name="Device Template" sheetId="2" r:id="rId4"/>
+    <sheet name="S7 Template" sheetId="10" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="131">
   <si>
     <t>HMI_TAG</t>
   </si>
@@ -357,38 +369,77 @@
     <t>mm</t>
   </si>
   <si>
+    <t>PLC</t>
+  </si>
+  <si>
+    <t>Group1</t>
+  </si>
+  <si>
+    <t>device_2</t>
+  </si>
+  <si>
+    <t>device_3</t>
+  </si>
+  <si>
     <t>device_1</t>
   </si>
   <si>
-    <t>Device #1 -</t>
-  </si>
-  <si>
-    <t>PLC</t>
-  </si>
-  <si>
-    <t>Group1</t>
-  </si>
-  <si>
-    <t>Device Template</t>
-  </si>
-  <si>
-    <t>device_2</t>
-  </si>
-  <si>
-    <t>device_3</t>
-  </si>
-  <si>
-    <t>Device #2 -</t>
-  </si>
-  <si>
-    <t>Device #3 -</t>
+    <t>HMI_TAG_real</t>
+  </si>
+  <si>
+    <t>COMMENT001 Real</t>
+  </si>
+  <si>
+    <t>OFFSET</t>
+  </si>
+  <si>
+    <t>PLC_TAG,XOFFSET.0</t>
+  </si>
+  <si>
+    <t>DB61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device 1 - </t>
+  </si>
+  <si>
+    <t>S7 Template</t>
+  </si>
+  <si>
+    <t>Device 2 -</t>
+  </si>
+  <si>
+    <t>Device 3 -</t>
+  </si>
+  <si>
+    <t>HMI_TAG_bit0</t>
+  </si>
+  <si>
+    <t>COMMENT001 Bit0</t>
+  </si>
+  <si>
+    <t>HMI_TAG_bit1</t>
+  </si>
+  <si>
+    <t>HMI_TAG_bit2</t>
+  </si>
+  <si>
+    <t>COMMENT001 Bit1</t>
+  </si>
+  <si>
+    <t>COMMENT001 Bit2</t>
+  </si>
+  <si>
+    <t>PLC_TAG,XOFFSET.1</t>
+  </si>
+  <si>
+    <t>PLC_TAG,XOFFSET.2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -412,6 +463,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -727,18 +784,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FF7939-21C8-4DCD-BC56-2BF400B9C3F2}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -757,65 +814,77 @@
       <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="G1" s="4" t="s">
+        <v>116</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D2" t="s">
         <v>109</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" t="s">
         <v>109</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E3" t="s">
         <v>110</v>
       </c>
-      <c r="D2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>112</v>
       </c>
-      <c r="F2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>115</v>
-      </c>
       <c r="B4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
+        <v>120</v>
+      </c>
+      <c r="G4">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2447,4 +2516,974 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{828F62E6-0D5B-4ABE-8C1D-379E50AD1A31}">
+  <dimension ref="A1:BL8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.7109375" customWidth="1"/>
+    <col min="43" max="43" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:64" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" t="s">
+        <v>85</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" t="s">
+        <v>27</v>
+      </c>
+      <c r="P3" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:64" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="W5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="X5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AH5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AJ5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="AK5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="AM5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AO5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP5" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AT5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AU5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="AV5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="AW5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="AX5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="AY5" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AZ5" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="BA5" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="BB5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="BC5" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="BD5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="BE5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="BF5" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="BG5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="BH5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="BI5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="BJ5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK5" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:64" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0</v>
+      </c>
+      <c r="M6" s="3">
+        <v>-32768</v>
+      </c>
+      <c r="N6" s="3">
+        <v>32767</v>
+      </c>
+      <c r="O6" s="3">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R6" s="3">
+        <v>0</v>
+      </c>
+      <c r="S6" s="3">
+        <v>1</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="U6" s="3">
+        <v>0</v>
+      </c>
+      <c r="V6" s="3">
+        <v>1</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AF6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AI6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AK6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="3">
+        <v>1</v>
+      </c>
+      <c r="AM6" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="AN6" s="3">
+        <v>-32768</v>
+      </c>
+      <c r="AO6" s="3">
+        <v>32767</v>
+      </c>
+      <c r="AP6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>31</v>
+      </c>
+      <c r="AR6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AT6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AV6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AY6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="3">
+        <v>0</v>
+      </c>
+      <c r="BA6" s="3">
+        <v>0</v>
+      </c>
+      <c r="BB6" s="3">
+        <v>0</v>
+      </c>
+      <c r="BC6" s="3">
+        <v>0</v>
+      </c>
+      <c r="BL6" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" t="s">
+        <v>40</v>
+      </c>
+      <c r="O7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S7" t="s">
+        <v>45</v>
+      </c>
+      <c r="T7" t="s">
+        <v>46</v>
+      </c>
+      <c r="U7" t="s">
+        <v>47</v>
+      </c>
+      <c r="V7" t="s">
+        <v>48</v>
+      </c>
+      <c r="W7" t="s">
+        <v>49</v>
+      </c>
+      <c r="X7" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>62</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>64</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>19</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AU7" t="s">
+        <v>21</v>
+      </c>
+      <c r="AV7" t="s">
+        <v>22</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>69</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>70</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>71</v>
+      </c>
+      <c r="AZ7" t="s">
+        <v>72</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>73</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>74</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>75</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>76</v>
+      </c>
+      <c r="BE7" t="s">
+        <v>77</v>
+      </c>
+      <c r="BF7" t="s">
+        <v>78</v>
+      </c>
+      <c r="BG7" t="s">
+        <v>79</v>
+      </c>
+      <c r="BH7" t="s">
+        <v>80</v>
+      </c>
+      <c r="BI7" t="s">
+        <v>81</v>
+      </c>
+      <c r="BJ7" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3"/>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" s="3">
+        <v>-32768</v>
+      </c>
+      <c r="N8" s="3">
+        <v>32767</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0.1</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>28</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>1</v>
+      </c>
+      <c r="T8" t="s">
+        <v>28</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>1</v>
+      </c>
+      <c r="W8" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+      <c r="AE8">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG8">
+        <v>0</v>
+      </c>
+      <c r="AH8">
+        <v>1</v>
+      </c>
+      <c r="AI8">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AK8">
+        <v>0</v>
+      </c>
+      <c r="AL8">
+        <v>1</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>83</v>
+      </c>
+      <c r="AN8" s="3">
+        <v>-32768</v>
+      </c>
+      <c r="AO8" s="3">
+        <v>32767</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>84</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>31</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AT8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AV8">
+        <v>0</v>
+      </c>
+      <c r="AW8">
+        <v>0</v>
+      </c>
+      <c r="AX8">
+        <v>0</v>
+      </c>
+      <c r="AY8">
+        <v>0</v>
+      </c>
+      <c r="AZ8">
+        <v>0</v>
+      </c>
+      <c r="BA8">
+        <v>0</v>
+      </c>
+      <c r="BB8">
+        <v>0</v>
+      </c>
+      <c r="BC8">
+        <v>0</v>
+      </c>
+      <c r="BL8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated OFFSET placeholder to {OFFSET+N} for readability. version 0.3.1
</commit_message>
<xml_diff>
--- a/ww_tag_template.xlsx
+++ b/ww_tag_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\wwtags\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCE7247-BA9C-4AB6-A54B-C63A44EFDB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6487FE4-30D8-40E9-8078-446A2B0BBDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="133">
   <si>
     <t>HMI_TAG</t>
   </si>
@@ -393,24 +393,12 @@
     <t>OFFSET</t>
   </si>
   <si>
-    <t>PLC_TAG,XOFFSET.0</t>
-  </si>
-  <si>
     <t>DB61</t>
   </si>
   <si>
-    <t xml:space="preserve">Device 1 - </t>
-  </si>
-  <si>
     <t>S7 Template</t>
   </si>
   <si>
-    <t>Device 2 -</t>
-  </si>
-  <si>
-    <t>Device 3 -</t>
-  </si>
-  <si>
     <t>HMI_TAG_bit0</t>
   </si>
   <si>
@@ -429,10 +417,28 @@
     <t>COMMENT001 Bit2</t>
   </si>
   <si>
-    <t>PLC_TAG,XOFFSET.1</t>
-  </si>
-  <si>
-    <t>PLC_TAG,XOFFSET.2</t>
+    <t>PLC_TAG,X{OFFSET+0}.0</t>
+  </si>
+  <si>
+    <t>PLC_TAG,X{OFFSET+0}.1</t>
+  </si>
+  <si>
+    <t>PLC_TAG,X{OFFSET+0}.2</t>
+  </si>
+  <si>
+    <t>PLC_TAG,INT{OFFSET+2}</t>
+  </si>
+  <si>
+    <t>PLC_TAG,REAL{OFFSET+4}</t>
+  </si>
+  <si>
+    <t>Device 1</t>
+  </si>
+  <si>
+    <t>Device 2</t>
+  </si>
+  <si>
+    <t>Device 3</t>
   </si>
 </sst>
 </file>
@@ -823,10 +829,10 @@
         <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
         <v>109</v>
@@ -835,7 +841,7 @@
         <v>110</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G2">
         <v>20</v>
@@ -846,10 +852,10 @@
         <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
         <v>109</v>
@@ -858,7 +864,7 @@
         <v>110</v>
       </c>
       <c r="F3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G3">
         <v>60</v>
@@ -869,10 +875,10 @@
         <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="D4" t="s">
         <v>109</v>
@@ -881,7 +887,7 @@
         <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G4">
         <v>100</v>
@@ -2529,7 +2535,7 @@
     <col min="14" max="14" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="24.7109375" customWidth="1"/>
     <col min="43" max="43" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="21.5703125" customWidth="1"/>
+    <col min="45" max="45" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:64" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2602,13 +2608,13 @@
     </row>
     <row r="2" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
         <v>27</v>
@@ -2647,7 +2653,7 @@
         <v>27</v>
       </c>
       <c r="P2" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="Q2" t="s">
         <v>27</v>
@@ -2661,13 +2667,13 @@
     </row>
     <row r="3" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
@@ -2706,7 +2712,7 @@
         <v>27</v>
       </c>
       <c r="P3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="Q3" t="s">
         <v>27</v>
@@ -2720,13 +2726,13 @@
     </row>
     <row r="4" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D4" t="s">
         <v>27</v>
@@ -2765,7 +2771,7 @@
         <v>27</v>
       </c>
       <c r="P4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="Q4" t="s">
         <v>27</v>
@@ -3098,6 +3104,9 @@
       <c r="AR6" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="AS6" t="s">
+        <v>128</v>
+      </c>
       <c r="AT6" s="3" t="s">
         <v>27</v>
       </c>
@@ -3450,6 +3459,9 @@
       </c>
       <c r="AR8" t="s">
         <v>27</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>129</v>
       </c>
       <c r="AT8" t="s">
         <v>27</v>

</xml_diff>